<commit_message>
Add dated configuration checkpoints and automatic PDF builds; retire PTC-X
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R4fd4afc41cf944e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="2" r:id="Rb160c8f52add41ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="3" r:id="Rc066ef1603194c26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="4" r:id="R5948c8af134446ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal spans" sheetId="5" r:id="R7ca8a6201c5d4062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluids" sheetId="6" r:id="Ra14d2b1473d1488a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="7" r:id="Ra0b132a87e9947d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model choices" sheetId="8" r:id="Rb3dcaa9871fe421b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form pipe" sheetId="9" r:id="Rbd1beffc2d7d4f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form sensor" sheetId="10" r:id="R9cdf0136f50a449e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form material" sheetId="11" r:id="Raf88f99e746a4296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="12" r:id="Rf133fd7bc31040a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase requests" sheetId="13" r:id="Rbc3cd00ee05f4c94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review issues" sheetId="14" r:id="R18074aadc6c14b1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R079a58e935414fe5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R3d2f3e7467d64bff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="2" r:id="R6ca0c0b358174654"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="3" r:id="Rcd6a7b01ec60446f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="4" r:id="Raa4e924a0d4b4380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal spans" sheetId="5" r:id="R95557c7300554084"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluids" sheetId="6" r:id="Rd1a195450d0244f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="7" r:id="R3e74bcec881d4e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model choices" sheetId="8" r:id="Rd8f76f5a2f7d42a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form pipe" sheetId="9" r:id="R041235539c544b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form sensor" sheetId="10" r:id="R44dff52537404fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form material" sheetId="11" r:id="Rca46a8c6c1d745b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="12" r:id="Rfab6aefbf3614370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase requests" sheetId="13" r:id="R577337ec05494dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review issues" sheetId="14" r:id="R38d66bb972ee4719"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rfabdf3b6caae4c4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -497,7 +497,7 @@
         <x:v>Configuration ID</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>VCU-REV9-DRAFT-001</x:v>
+        <x:v>VCU-REV9-DRAFT-002</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Change after physical configuration changes.</x:v>
@@ -625,7 +625,7 @@
         <x:v>Output refresh</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>Package maintainer: see START_HERE.md</x:v>
+        <x:v>Upload to GitHub; Actions builds the PDF. See support/docs/DATED_CHECKPOINTS.md.</x:v>
       </x:c>
       <x:c r="C19" s="8" t="str">
         <x:v>The experimental team can complete forms without running scripts.</x:v>
@@ -651,6 +651,28 @@
       </x:c>
       <x:c r="C21" s="8" t="str">
         <x:v>Assign the circuit and operating range for each experiment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="9" t="str">
+        <x:v>Effective date</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C22" s="9" t="str">
+        <x:v>Date this documentation configuration takes effect; ISO YYYY-MM-DD text.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="64" customHeight="1">
+      <x:c r="A23" s="9" t="str">
+        <x:v>Change summary</x:v>
+      </x:c>
+      <x:c r="B23" s="9" t="str">
+        <x:v>PTC-X removed from active sensor and calibration records at the repository owner's request. Documentation change only; no physical removal or installed-hardware verification is asserted.</x:v>
+      </x:c>
+      <x:c r="C23" s="9" t="str">
+        <x:v>Describe changes since the preceding configuration and identify evidence or the request.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1790,19 +1812,19 @@
         <x:v>Campaign execution conventions; proposed revision log</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>2026-10-16 / VCU-REV9-DRAFT-002: PTC-X removed from active sensor and calibration records at the repository owner's request. Documentation change only; no physical removal or installed-hardware verification is asserted.</x:v>
       </x:c>
       <x:c r="J7" s="17" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Reported</x:v>
       </x:c>
       <x:c r="K7" s="17" t="str">
-        <x:v>None supplied</x:v>
+        <x:v>USER</x:v>
       </x:c>
       <x:c r="L7" s="17" t="str">
-        <x:v>Not available</x:v>
+        <x:v>Repository owner request in the Codex session, 2026-10-16; Start effective date and change summary.</x:v>
       </x:c>
       <x:c r="M7" s="17" t="str">
-        <x:v>Needs information</x:v>
+        <x:v>Needs review</x:v>
       </x:c>
       <x:c r="N7" s="17" t="str">
         <x:v>Record effective date, author, changed item, reason, previous/new evidence, affected runs and whether recalibration or model revalidation is needed.</x:v>
@@ -2717,7 +2739,7 @@
         <x:v>Needs review</x:v>
       </x:c>
       <x:c r="N26" s="17" t="str">
-        <x:v>Confirm installed count and resolve PTC-X; no channel identity inferred.</x:v>
+        <x:v>Verify installed hardware count and channel identities for remaining sensors. PTC-X was removed from the active register at the repository owner's request on 2026-10-16; no physical removal is asserted.</x:v>
       </x:c>
       <x:c r="O26" s="19"/>
       <x:c r="P26" s="19"/>
@@ -5468,7 +5490,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c4af1978db4fbd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2093fdc13f34801"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5631,7 +5653,7 @@
         <x:v>P0 Method: instrumentation</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>Resolve PTC-X; do not copy CAD IDs or assume TC/Luna co-location.</x:v>
+        <x:v>PTC-X omitted from the active register by owner request, 2026-10-16. Verify remaining installed sensor identities; do not assume CAD IDs are DAQ channels or TC/Luna co-location.</x:v>
       </x:c>
       <x:c r="J7" s="17" t="str">
         <x:v>Evidence supplied and reviewed; open limitations recorded.</x:v>
@@ -6120,7 +6142,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd89ff63fa3604e25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5944131610884552"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6281,13 +6303,13 @@
         <x:v>R9 sheets 5-6; SNOTE VCU Rev9 PTCX note</x:v>
       </x:c>
       <x:c r="D9" s="17" t="str">
-        <x:v>CAD extraction includes PTC-X; note calls PTCX a fluke.</x:v>
+        <x:v>Historical CAD extraction includes PTC-X; the supplied note calls PTCX a fluke. PTC-X was removed from the active sensor/calibration records by owner request, 2026-10-16. Installed hardware identity is unverified.</x:v>
       </x:c>
       <x:c r="E9" s="17" t="str">
         <x:v>Experimental instrumentation</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>Check installed hardware and source labeling; keep unresolved reference until dispositioned.</x:v>
+        <x:v>Retain the original CAD/source evidence. Confirm whether the excluded reference corresponds to installed hardware before using it in any run or model mapping.</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">
         <x:v>C21; C23</x:v>
@@ -6411,7 +6433,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a88f358128c49c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab575658e8534009"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6768,7 +6790,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R368ebb592a1a4c9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R866c82e6ea2645b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7803,36 +7825,18 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="26" customHeight="1">
-      <x:c r="A21" s="8" t="str">
-        <x:v>PTC-X</x:v>
-      </x:c>
-      <x:c r="B21" s="8" t="str">
-        <x:v>PTC</x:v>
-      </x:c>
-      <x:c r="C21" s="8" t="str">
-        <x:v>downcomer</x:v>
-      </x:c>
-      <x:c r="D21" s="8" t="str">
-        <x:v>G</x:v>
-      </x:c>
-      <x:c r="E21" s="10" t="n">
-        <x:v>50.799998652460545</x:v>
-      </x:c>
+      <x:c r="A21" s="8"/>
+      <x:c r="B21" s="8"/>
+      <x:c r="C21" s="8"/>
+      <x:c r="D21" s="8"/>
+      <x:c r="E21" s="10"/>
       <x:c r="F21" s="10"/>
       <x:c r="G21" s="10"/>
       <x:c r="H21" s="8"/>
-      <x:c r="I21" s="8" t="str">
-        <x:v>CAD-derived</x:v>
-      </x:c>
-      <x:c r="J21" s="8" t="str">
-        <x:v>Mount reference</x:v>
-      </x:c>
-      <x:c r="K21" s="8" t="str">
-        <x:v>VCU-R9-E01 (2026-10-08) sheets 5-7</x:v>
-      </x:c>
-      <x:c r="L21" s="8" t="str">
-        <x:v>Conflicts with note: PTCX is a fluke; verify installed hardware.</x:v>
-      </x:c>
+      <x:c r="I21" s="8"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="8"/>
+      <x:c r="L21" s="8"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="8" t="str">
@@ -8397,9 +8401,7 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="26" customHeight="1">
-      <x:c r="A21" s="8" t="str">
-        <x:v>PTC-X</x:v>
-      </x:c>
+      <x:c r="A21" s="8"/>
       <x:c r="B21" s="8"/>
       <x:c r="C21" s="8"/>
       <x:c r="D21" s="8"/>
@@ -8410,9 +8412,7 @@
       <x:c r="I21" s="8"/>
       <x:c r="J21" s="8"/>
       <x:c r="K21" s="8"/>
-      <x:c r="L21" s="8" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
+      <x:c r="L21" s="8"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="8" t="str">

</xml_diff>

<commit_message>
Add workbook-controlled insulation coverage diagrams and exports
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -2,21 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="R3d2f3e7467d64bff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="2" r:id="R6ca0c0b358174654"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="3" r:id="Rcd6a7b01ec60446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="4" r:id="Raa4e924a0d4b4380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal spans" sheetId="5" r:id="R95557c7300554084"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluids" sheetId="6" r:id="Rd1a195450d0244f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="7" r:id="R3e74bcec881d4e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model choices" sheetId="8" r:id="Rd8f76f5a2f7d42a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form pipe" sheetId="9" r:id="R041235539c544b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form sensor" sheetId="10" r:id="R44dff52537404fc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form material" sheetId="11" r:id="Rca46a8c6c1d745b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="12" r:id="Rfab6aefbf3614370"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase requests" sheetId="13" r:id="R577337ec05494dd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review issues" sheetId="14" r:id="R38d66bb972ee4719"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="Rfabdf3b6caae4c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="Rdb02ed5692054212"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="2" r:id="Rf1a1c2c29ae74f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="3" r:id="R8cf742f24a1242b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="4" r:id="Rce9e1ed27a584c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal spans" sheetId="5" r:id="R71573f0f7a2441c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluids" sheetId="6" r:id="R1ed7dc31f52e48ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="7" r:id="R9eb6acc318f84a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model choices" sheetId="8" r:id="R7829d47b1a094173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form pipe" sheetId="9" r:id="R8e46e6eef5be4265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form sensor" sheetId="10" r:id="R0033565f60de4b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form material" sheetId="11" r:id="R22ed0c6c434a4896"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="12" r:id="R187ac51e51ea41b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase requests" sheetId="13" r:id="Rcd7df112b25b46dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review issues" sheetId="14" r:id="Rdade0e14c7f84263"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R598c4ac295604744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insulation regions" sheetId="16" r:id="R0557123f889541bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27,10 +28,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="200" formatCode="0.000"/>
+    <x:numFmt numFmtId="201" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +66,25 @@
       <x:color rgb="FF576976"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF203D4C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -97,6 +116,21 @@
         <x:fgColor rgb="FFFFF4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF16374A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF3F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -110,7 +144,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="35">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -166,6 +200,41 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -497,7 +566,7 @@
         <x:v>Configuration ID</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>VCU-REV9-DRAFT-002</x:v>
+        <x:v>VCU-REV9-DRAFT-003</x:v>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Change after physical configuration changes.</x:v>
@@ -614,7 +683,7 @@
         <x:v>Editing sequence</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
-        <x:v>Start with Form pipe, Form sensor and Form material</x:v>
+        <x:v>Start with Form tabs, or Insulation regions for whole-region coverage.</x:v>
       </x:c>
       <x:c r="C18" s="8" t="str">
         <x:v>Read the reference; enter new evidence in amber cells; send for review.</x:v>
@@ -669,7 +738,7 @@
         <x:v>Change summary</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>PTC-X removed from active sensor and calibration records at the repository owner's request. Documentation change only; no physical removal or installed-hardware verification is asserted.</x:v>
+        <x:v>Added ten insulation regions, coverage dropdowns and a separate diagram. All coverage starts Unknown pending evidence. PTC-X remains excluded from the active register.</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
         <x:v>Describe changes since the preceding configuration and identify evidence or the request.</x:v>
@@ -1812,7 +1881,7 @@
         <x:v>Campaign execution conventions; proposed revision log</x:v>
       </x:c>
       <x:c r="I7" s="17" t="str">
-        <x:v>2026-10-16 / VCU-REV9-DRAFT-002: PTC-X removed from active sensor and calibration records at the repository owner's request. Documentation change only; no physical removal or installed-hardware verification is asserted.</x:v>
+        <x:v>2026-10-16 / VCU-REV9-DRAFT-002: PTC-X removed from active sensor and calibration records at the repository owner's request. Documentation change only; no physical removal or installed-hardware verification is asserted. 2026-10-16 / VCU-REV9-DRAFT-003: added ten insulation coverage regions and the diagram; all coverage Unknown pending evidence.</x:v>
       </x:c>
       <x:c r="J7" s="17" t="str">
         <x:v>Reported</x:v>
@@ -1821,7 +1890,7 @@
         <x:v>USER</x:v>
       </x:c>
       <x:c r="L7" s="17" t="str">
-        <x:v>Repository owner request in the Codex session, 2026-10-16; Start effective date and change summary.</x:v>
+        <x:v>Start effective date and change summary; previous record saved at support/checkpoints/2026-10-16_VCU-REV9-DRAFT-002/. Owner-approved insulation feature plan in the Codex session, 2026-10-16; installed coverage remains unconfirmed.</x:v>
       </x:c>
       <x:c r="M7" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -5490,7 +5559,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2093fdc13f34801"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe3645e732ce4448"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6142,7 +6211,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5944131610884552"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4efd2b3592534634"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6433,7 +6502,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab575658e8534009"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9e02aec8f064b4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6790,8 +6859,402 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R866c82e6ea2645b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd789b6a13c34804"/>
   </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="56" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="42" customHeight="1">
+      <x:c r="A1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="B1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="C1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="D1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="F1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="G1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="H1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+      <x:c r="I1" s="29" t="str">
+        <x:v>Insulation coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="29" customHeight="1">
+      <x:c r="A2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="B2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="C2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="D2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="E2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="F2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="G2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="H2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+      <x:c r="I2" s="30" t="str">
+        <x:v>Choose Unknown, Insulated or Bare for each whole region. Gray cells identify the region; amber cells are editable.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="29" customHeight="1">
+      <x:c r="A3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="B3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="C3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="D3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="E3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="F3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="G3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="H3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+      <x:c r="I3" s="30" t="str">
+        <x:v>Material ID refers to the Materials tab. Thickness is in mm. Add evidence and identify the insulated surface, particularly around the cooler jacket.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="29" customHeight="1">
+      <x:c r="A4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="B4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="C4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="D4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="E4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="F4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="G4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="H4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+      <x:c r="I4" s="30" t="str">
+        <x:v>Pre/post follow drawing traversal. Top boundaries come from Complete jacket on Thermal spans; corners are schematic. Upload the workbook to rebuild the PDF.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="31" t="str">
+        <x:v>Region ID</x:v>
+      </x:c>
+      <x:c r="B5" s="31" t="str">
+        <x:v>Region</x:v>
+      </x:c>
+      <x:c r="C5" s="31" t="str">
+        <x:v>Boundary reference</x:v>
+      </x:c>
+      <x:c r="D5" s="31" t="str">
+        <x:v>Coverage</x:v>
+      </x:c>
+      <x:c r="E5" s="31" t="str">
+        <x:v>Material ID</x:v>
+      </x:c>
+      <x:c r="F5" s="31" t="str">
+        <x:v>Thickness mm</x:v>
+      </x:c>
+      <x:c r="G5" s="31" t="str">
+        <x:v>Evidence type</x:v>
+      </x:c>
+      <x:c r="H5" s="31" t="str">
+        <x:v>Evidence file / location</x:v>
+      </x:c>
+      <x:c r="I5" s="31" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="54" customHeight="1">
+      <x:c r="A6" s="32" t="str">
+        <x:v>INS-01</x:v>
+      </x:c>
+      <x:c r="B6" s="32" t="str">
+        <x:v>Upcomer</x:v>
+      </x:c>
+      <x:c r="C6" s="32" t="str">
+        <x:v>Full segment</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E6" s="33"/>
+      <x:c r="F6" s="34"/>
+      <x:c r="G6" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H6" s="33"/>
+      <x:c r="I6" s="33"/>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" s="32" t="str">
+        <x:v>INS-02</x:v>
+      </x:c>
+      <x:c r="B7" s="32" t="str">
+        <x:v>Top-left corner</x:v>
+      </x:c>
+      <x:c r="C7" s="32" t="str">
+        <x:v>Full schematic corner</x:v>
+      </x:c>
+      <x:c r="D7" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E7" s="33"/>
+      <x:c r="F7" s="34"/>
+      <x:c r="G7" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H7" s="33"/>
+      <x:c r="I7" s="33"/>
+    </x:row>
+    <x:row r="8" ht="54" customHeight="1">
+      <x:c r="A8" s="32" t="str">
+        <x:v>INS-03</x:v>
+      </x:c>
+      <x:c r="B8" s="32" t="str">
+        <x:v>Pre-cooler</x:v>
+      </x:c>
+      <x:c r="C8" s="32" t="str">
+        <x:v>Segment start to Complete jacket start</x:v>
+      </x:c>
+      <x:c r="D8" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E8" s="33"/>
+      <x:c r="F8" s="34"/>
+      <x:c r="G8" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H8" s="33"/>
+      <x:c r="I8" s="33"/>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" s="32" t="str">
+        <x:v>INS-04</x:v>
+      </x:c>
+      <x:c r="B9" s="32" t="str">
+        <x:v>Cooler</x:v>
+      </x:c>
+      <x:c r="C9" s="32" t="str">
+        <x:v>Complete jacket start to Complete jacket end</x:v>
+      </x:c>
+      <x:c r="D9" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E9" s="33"/>
+      <x:c r="F9" s="34"/>
+      <x:c r="G9" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H9" s="33"/>
+      <x:c r="I9" s="33" t="str">
+        <x:v>Identify the insulated surface, especially jacket exterior versus pipe.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" s="32" t="str">
+        <x:v>INS-05</x:v>
+      </x:c>
+      <x:c r="B10" s="32" t="str">
+        <x:v>Post-cooler</x:v>
+      </x:c>
+      <x:c r="C10" s="32" t="str">
+        <x:v>Complete jacket end to segment end</x:v>
+      </x:c>
+      <x:c r="D10" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E10" s="33"/>
+      <x:c r="F10" s="34"/>
+      <x:c r="G10" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H10" s="33"/>
+      <x:c r="I10" s="33"/>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" s="32" t="str">
+        <x:v>INS-06</x:v>
+      </x:c>
+      <x:c r="B11" s="32" t="str">
+        <x:v>Top-right corner</x:v>
+      </x:c>
+      <x:c r="C11" s="32" t="str">
+        <x:v>Full schematic corner</x:v>
+      </x:c>
+      <x:c r="D11" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E11" s="33"/>
+      <x:c r="F11" s="34"/>
+      <x:c r="G11" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H11" s="33"/>
+      <x:c r="I11" s="33"/>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" s="32" t="str">
+        <x:v>INS-07</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>Downcomer</x:v>
+      </x:c>
+      <x:c r="C12" s="32" t="str">
+        <x:v>Full segment</x:v>
+      </x:c>
+      <x:c r="D12" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E12" s="33"/>
+      <x:c r="F12" s="34"/>
+      <x:c r="G12" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H12" s="33"/>
+      <x:c r="I12" s="33"/>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" s="32" t="str">
+        <x:v>INS-08</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>Bottom-right corner</x:v>
+      </x:c>
+      <x:c r="C13" s="32" t="str">
+        <x:v>Full schematic corner</x:v>
+      </x:c>
+      <x:c r="D13" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E13" s="33"/>
+      <x:c r="F13" s="34"/>
+      <x:c r="G13" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H13" s="33"/>
+      <x:c r="I13" s="33"/>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" s="32" t="str">
+        <x:v>INS-09</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="str">
+        <x:v>Heater</x:v>
+      </x:c>
+      <x:c r="C14" s="32" t="str">
+        <x:v>Full segment</x:v>
+      </x:c>
+      <x:c r="D14" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E14" s="33"/>
+      <x:c r="F14" s="34"/>
+      <x:c r="G14" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H14" s="33"/>
+      <x:c r="I14" s="33"/>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" s="32" t="str">
+        <x:v>INS-10</x:v>
+      </x:c>
+      <x:c r="B15" s="32" t="str">
+        <x:v>Bottom-left corner</x:v>
+      </x:c>
+      <x:c r="C15" s="32" t="str">
+        <x:v>Full schematic corner</x:v>
+      </x:c>
+      <x:c r="D15" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="E15" s="33"/>
+      <x:c r="F15" s="34"/>
+      <x:c r="G15" s="33" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="H15" s="33"/>
+      <x:c r="I15" s="33"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A3:I3"/>
+    <x:mergeCell ref="A4:I4"/>
+  </x:mergeCells>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="D6:D15">
+      <x:formula1>"Unknown,Insulated,Bare"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G6:G15">
+      <x:formula1>"Unknown,CAD-derived,Installed measurement,Reported,Modeling assumption"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="decimal" operator="greaterThanOrEqual" sqref="F6:F15">
+      <x:formula1>0</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add traceable VCU geometry and material references to draft configuration
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start" sheetId="1" r:id="Rdb02ed5692054212"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry" sheetId="2" r:id="Rf1a1c2c29ae74f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="3" r:id="R8cf742f24a1242b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration" sheetId="4" r:id="Rce9e1ed27a584c06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thermal spans" sheetId="5" r:id="R71573f0f7a2441c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluids" sheetId="6" r:id="R1ed7dc31f52e48ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="7" r:id="R9eb6acc318f84a13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model choices" sheetId="8" r:id="R7829d47b1a094173"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form pipe" sheetId="9" r:id="R8e46e6eef5be4265"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form sensor" sheetId="10" r:id="R0033565f60de4b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form material" sheetId="11" r:id="R22ed0c6c434a4896"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="12" r:id="R187ac51e51ea41b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase requests" sheetId="13" r:id="Rcd7df112b25b46dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review issues" sheetId="14" r:id="Rdade0e14c7f84263"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" r:id="R598c4ac295604744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insulation regions" sheetId="16" r:id="R0557123f889541bd"/>
+    <x:sheet name="Start" sheetId="1" r:id="Rdb02ed5692054212"/>
+    <x:sheet name="Geometry" sheetId="2" r:id="Rf1a1c2c29ae74f1d"/>
+    <x:sheet name="Sensors" sheetId="3" r:id="R8cf742f24a1242b4"/>
+    <x:sheet name="Calibration" sheetId="4" r:id="Rce9e1ed27a584c06"/>
+    <x:sheet name="Thermal spans" sheetId="5" r:id="R71573f0f7a2441c6"/>
+    <x:sheet name="Fluids" sheetId="6" r:id="R1ed7dc31f52e48ce"/>
+    <x:sheet name="Materials" sheetId="7" r:id="R9eb6acc318f84a13"/>
+    <x:sheet name="Model choices" sheetId="8" r:id="R7829d47b1a094173"/>
+    <x:sheet name="Form pipe" sheetId="9" r:id="R8e46e6eef5be4265"/>
+    <x:sheet name="Form sensor" sheetId="10" r:id="R0033565f60de4b42"/>
+    <x:sheet name="Form material" sheetId="11" r:id="R22ed0c6c434a4896"/>
+    <x:sheet name="Requirements" sheetId="12" r:id="R187ac51e51ea41b6"/>
+    <x:sheet name="Phase requests" sheetId="13" r:id="Rcd7df112b25b46dd"/>
+    <x:sheet name="Review issues" sheetId="14" r:id="Rdade0e14c7f84263"/>
+    <x:sheet name="Sources" sheetId="15" r:id="R598c4ac295604744"/>
+    <x:sheet name="Insulation regions" sheetId="16" r:id="R0557123f889541bd"/>
+    <x:sheet name="CAD dimensions" sheetId="17" r:id="rIdCFG001Dimensions"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,6 +507,470 @@
 </a:theme>
 </file>
 
+<file path=xl/worksheets/cfg001_dimensions.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="86" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="112" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="11" t="inlineStr">
+        <x:is>
+          <x:t>VCU Rev9 component reference dimensions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="11"/>
+      <x:c r="C1" s="11"/>
+      <x:c r="D1" s="11"/>
+      <x:c r="E1" s="11"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="12" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived local dimensions; not installed measurements. Main bore unknown.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="13" t="inlineStr">
+        <x:is>
+          <x:t>Use local bores only for the identified component. Portable source: support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="11"/>
+      <x:c r="C3" s="11"/>
+      <x:c r="D3" s="11"/>
+      <x:c r="E3" s="11"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="11"/>
+      <x:c r="B4" s="11"/>
+      <x:c r="C4" s="11"/>
+      <x:c r="D4" s="11"/>
+      <x:c r="E4" s="11"/>
+    </x:row>
+    <x:row r="5" ht="44" customHeight="1">
+      <x:c r="A5" s="16" t="inlineStr">
+        <x:is>
+          <x:t>Record ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="16" t="inlineStr">
+        <x:is>
+          <x:t>Component</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="16" t="inlineStr">
+        <x:is>
+          <x:t>Reference values</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="16" t="inlineStr">
+        <x:is>
+          <x:t>Units</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="16" t="inlineStr">
+        <x:is>
+          <x:t>Evidence / limitations</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="110" customHeight="1">
+      <x:c r="A6" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-01</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Main swept loop</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=33.401</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Main swept loop; Both main-loop definitions have only the outer pipe envelope. Main bore absent.; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="110" customHeight="1">
+      <x:c r="A7" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-02</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="17" t="inlineStr">
+        <x:is>
+          <x:t>TLEP / BREP</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=33.401; inner_diameter_mm=26.924; wall_thickness_mm=3.238500000000002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / TLEP / BREP; Annular exit tube cylinders; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F2 / F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="110" customHeight="1">
+      <x:c r="A8" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-03</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Cooling jacket shell</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=88.9; inner_diameter_mm=77.9272; wall_thickness_mm=5.486400000000003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Cooling jacket shell; Concentric shell cylinders; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F4 / F3</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="110" customHeight="1">
+      <x:c r="A9" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Jacket end plates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=88.9; inner_diameter_mm=33.655; radial_width_mm=27.622500000000002; axial_thickness_mm=6.35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Jacket end plates; Inner diameter is the pipe clearance hole, not coolant-annulus diameter; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F2 / F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="110" customHeight="1">
+      <x:c r="A10" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Jacket port nipples</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=33.401; inner_diameter_mm=26.6446; wall_thickness_mm=3.3782000000000014</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Jacket port nipples; OD is cylindrical land; thread shape is not represented by this value; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F1 / F27</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="110" customHeight="1">
+      <x:c r="A11" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-06</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="17" t="inlineStr">
+        <x:is>
+          <x:t>HX hoses</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=35.814</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / HX hoses; Solid swept envelope; hose bore absent; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="110" customHeight="1">
+      <x:c r="A12" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-07</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Drain-valve body</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=42.545; inner_diameter_mm=34.671; wall_thickness_mm=3.937000000000001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Drain-valve body; Simplified body, multiple intersecting cylinder spans; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F7 / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="110" customHeight="1">
+      <x:c r="A13" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-08</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="17" t="inlineStr">
+        <x:is>
+          <x:t>LF / combined sensor spools</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=33.401; inner_diameter_mm=26.6446; wall_thickness_mm=3.3782000000000014</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / LF / combined sensor spools; Local spool dimensions; do not apply bore globally; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F5 / F4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="110" customHeight="1">
+      <x:c r="A14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-09</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>PTC / JTC mount spools</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=33.528; inner_diameter_mm=25.4; wall_thickness_mm=4.064</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / PTC / JTC mount spools; Local 76.2 mm spool; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F3 / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="110" customHeight="1">
+      <x:c r="A15" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="17" t="inlineStr">
+        <x:is>
+          <x:t>TC sheath</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=3.175</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / TC sheath; External sheath only; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="110" customHeight="1">
+      <x:c r="A16" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="17" t="inlineStr">
+        <x:is>
+          <x:t>PTC guide tubing</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=6.35; inner_diameter_mm=4.572; wall_thickness_mm=0.8889999999999998</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / PTC guide tubing; Local instrument tubing; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F1 / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="110" customHeight="1">
+      <x:c r="A17" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="17" t="inlineStr">
+        <x:is>
+          <x:t>LF guide tubing</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=6.35; inner_diameter_mm=3.8608; wall_thickness_mm=1.2446</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / LF guide tubing; Local instrument tubing; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F1 / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="110" customHeight="1">
+      <x:c r="A18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Fiber capillary tubing</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=1.5875; inner_diameter_mm=1.0922; wall_thickness_mm=0.24764999999999993</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Fiber capillary tubing; Local optical capillary tubing; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F1 / F2</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="110" customHeight="1">
+      <x:c r="A19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIM-14</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Expansion tank shell</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>outer_diameter_mm=203.2; inner_diameter_mm=198.09378228810465; wall_thickness_mm=2.55310885594767</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD-derived; DIA / Expansion tank shell; Outer axial span 311.15 mm; support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Diameters.csv / F2 / F1</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart r:id="Rbd789b6a13c34804"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -565,8 +1030,10 @@
       <x:c r="A7" s="8" t="str">
         <x:v>Configuration ID</x:v>
       </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>VCU-REV9-DRAFT-003</x:v>
+      <x:c r="B7" s="9" t="inlineStr">
+        <x:is>
+          <x:t>VCU-REV9-DRAFT-004</x:t>
+        </x:is>
       </x:c>
       <x:c r="C7" s="8" t="str">
         <x:v>Change after physical configuration changes.</x:v>
@@ -664,7 +1131,11 @@
       <x:c r="A16" s="8" t="str">
         <x:v>Prepared by</x:v>
       </x:c>
-      <x:c r="B16" s="9"/>
+      <x:c r="B16" s="9" t="inlineStr">
+        <x:is>
+          <x:t>Codex; VCU reference synchronization requested by Andres Fierro</x:t>
+        </x:is>
+      </x:c>
       <x:c r="C16" s="8" t="str">
         <x:v>Enter name.</x:v>
       </x:c>
@@ -737,8 +1208,10 @@
       <x:c r="A23" s="9" t="str">
         <x:v>Change summary</x:v>
       </x:c>
-      <x:c r="B23" s="9" t="str">
-        <x:v>Added ten insulation regions, coverage dropdowns and a separate diagram. All coverage starts Unknown pending evidence. PTC-X remains excluded from the active register.</x:v>
+      <x:c r="B23" s="9" t="inlineStr">
+        <x:is>
+          <x:t>CFG-001: VCU Rev9 component dimensions; nine solid-property candidate functions with SI units and working domains; portable source copies; dated nominal-ID, insulation and heater assumptions in evidence records. Physical installation and approval remain open.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C23" s="9" t="str">
         <x:v>Describe changes since the preceding configuration and identify evidence or the request.</x:v>
@@ -1410,14 +1883,18 @@
       <x:c r="B9" s="17" t="str">
         <x:v>Input variable and output units</x:v>
       </x:c>
-      <x:c r="C9" s="18" t="str">
-        <x:v>Output W/(m K) reported; confirm T convention against original fit</x:v>
+      <x:c r="C9" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT candidate: T in K; k W/(m*K). Original fit temperature convention not independently verified.</x:t>
+        </x:is>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="E9" s="18" t="str">
-        <x:v>MAT lines 38-40</x:v>
+      <x:c r="E9" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; Materials MAIN-INS</x:t>
+        </x:is>
       </x:c>
       <x:c r="F9" s="19"/>
       <x:c r="G9" s="19"/>
@@ -1433,14 +1910,18 @@
       <x:c r="B10" s="17" t="str">
         <x:v>Source-supported domain</x:v>
       </x:c>
-      <x:c r="C10" s="18" t="str">
-        <x:v>Notes report 297-533 K; original data/domain unverified</x:v>
+      <x:c r="C10" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Original claimed k fit 297-533 K; user-authorized working extrapolation to 278.15 K (5 C), not product validation.</x:t>
+        </x:is>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="E10" s="18" t="str">
-        <x:v>MAT line 40</x:v>
+      <x:c r="E10" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C</x:t>
+        </x:is>
       </x:c>
       <x:c r="F10" s="19"/>
       <x:c r="G10" s="19"/>
@@ -1548,14 +2029,20 @@
       <x:c r="B15" s="17" t="str">
         <x:v>Interpolation and outside-domain policy</x:v>
       </x:c>
-      <x:c r="C15" s="18" t="str">
-        <x:v>Not selected</x:v>
-      </x:c>
-      <x:c r="D15" s="18" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E15" s="18" t="str">
-        <x:v>Proposed implementation record</x:v>
+      <x:c r="C15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT candidate: evaluate polynomial within working domain; error outside. No approved release implied.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT properties.conductivity</x:t>
+        </x:is>
       </x:c>
       <x:c r="F15" s="19"/>
       <x:c r="G15" s="19"/>
@@ -1594,14 +2081,20 @@
       <x:c r="B17" s="17" t="str">
         <x:v>Check values, implementation and version</x:v>
       </x:c>
-      <x:c r="C17" s="18" t="str">
-        <x:v>Not implemented or independently checked</x:v>
-      </x:c>
-      <x:c r="D17" s="18" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E17" s="18" t="str">
-        <x:v>Proposed property tests</x:v>
+      <x:c r="C17" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT v3 implementation candidate retained; portable coefficient transcription checks in CFG-001 report. Original data comparison remains open.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; CFG-001 report</x:t>
+        </x:is>
       </x:c>
       <x:c r="F17" s="19"/>
       <x:c r="G17" s="19"/>
@@ -1644,7 +2137,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
@@ -2216,17 +2709,23 @@
       <x:c r="H14" s="17" t="str">
         <x:v>Geometry map; Main swept loop</x:v>
       </x:c>
-      <x:c r="I14" s="17" t="str">
-        <x:v>Main CAD bore absent; notes report nominal 1.049 in (26.64 mm)</x:v>
+      <x:c r="I14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>CAD main bore absent. GEO-008 retains 26.64 mm rounded nominal ID for provisional main piping; not a CAD-extracted bore or installed measurement. Local spool bores differ.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J14" s="17" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K14" s="17" t="str">
-        <x:v>DIA; MAT</x:v>
-      </x:c>
-      <x:c r="L14" s="17" t="str">
-        <x:v>Main swept loop row; VCU Piping lines 23-27</x:v>
+      <x:c r="K14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>DIA; VSEL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L14" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Main swept loop; GEO-008 main nominal ID; CAD dimensions tab</x:t>
+        </x:is>
       </x:c>
       <x:c r="M14" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -2408,17 +2907,23 @@
       <x:c r="H18" s="17" t="str">
         <x:v>Geometry map; VCU insulation</x:v>
       </x:c>
-      <x:c r="I18" s="17" t="str">
-        <x:v>Main: fiberglass 5556K73; heater: calcium aluminum silicate 4057K14 reported</x:v>
+      <x:c r="I18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported fiberglass main insulation and calcium-aluminum-silicate heater strip. VINS v5 specifies regional candidates; product/installation evidence unresolved.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J18" s="17" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K18" s="17" t="str">
-        <x:v>MAT</x:v>
-      </x:c>
-      <x:c r="L18" s="17" t="str">
-        <x:v>Lines 29-44</x:v>
+      <x:c r="K18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>MAT; VINS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Materials; insulation.yaml regions; source copies in support/evidence/2026-10-16_CFG-001_vcu_references</x:t>
+        </x:is>
       </x:c>
       <x:c r="M18" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -2456,17 +2961,23 @@
       <x:c r="H19" s="17" t="str">
         <x:v>Geometry map; VCU insulation</x:v>
       </x:c>
-      <x:c r="I19" s="17" t="str">
-        <x:v>Most piping about 2 in; heater insulation 1/4 in reported</x:v>
+      <x:c r="I19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Approximate regional estimates: ordinary insulated pipe 50.8 mm fiberglass; heater 6.35 mm strip only. Top D-E is bare per GEO-008. Not measured thicknesses.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J19" s="17" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K19" s="17" t="str">
-        <x:v>MAT</x:v>
-      </x:c>
-      <x:c r="L19" s="17" t="str">
-        <x:v>Lines 29-44</x:v>
+      <x:c r="K19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VINS; VSEL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>insulation.yaml regions.non_heater_main_pipe and heater_leg; GEO-008 top-leg qualification</x:t>
+        </x:is>
       </x:c>
       <x:c r="M19" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -2504,20 +3015,30 @@
       <x:c r="H20" s="17" t="str">
         <x:v>Method: facility and fluid configuration; geometry map</x:v>
       </x:c>
-      <x:c r="I20" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="J20" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="K20" s="17" t="str">
-        <x:v>None supplied</x:v>
-      </x:c>
-      <x:c r="L20" s="17" t="str">
-        <x:v>Not available</x:v>
-      </x:c>
-      <x:c r="M20" s="17" t="str">
-        <x:v>Needs information</x:v>
+      <x:c r="I20" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 reports whole top D-E uninsulated; all STCs contact bare pipe locally. Remaining transition endpoints unknown. Older full-loop coverage text is superseded.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J20" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K20" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VSEL; VINS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L20" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 User direction and interpretation; insulation.yaml coverage</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M20" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N20" s="17" t="str">
         <x:v>Supply evidence and request review.</x:v>
@@ -2552,17 +3073,23 @@
       <x:c r="H21" s="17" t="str">
         <x:v>Geometry map; VCU Insulation</x:v>
       </x:c>
-      <x:c r="I21" s="17" t="str">
-        <x:v>Firm contact is explicitly an assumption in notes</x:v>
+      <x:c r="I21" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Perfect thermal contact is a user-directed model assumption (VINS), not a surveyed contact condition. Actual supports, gaps and layers remain open.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J21" s="17" t="str">
         <x:v>Modeling assumption</x:v>
       </x:c>
-      <x:c r="K21" s="17" t="str">
-        <x:v>HEAT</x:v>
-      </x:c>
-      <x:c r="L21" s="17" t="str">
-        <x:v>VCU Insulation lines 7-10</x:v>
+      <x:c r="K21" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VINS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L21" s="17" t="inlineStr">
+        <x:is>
+          <x:t>insulation.yaml contact</x:t>
+        </x:is>
       </x:c>
       <x:c r="M21" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -3416,17 +3943,25 @@
       <x:c r="H39" s="17" t="str">
         <x:v>Geometry map; heater note; sheet 4</x:v>
       </x:c>
-      <x:c r="I39" s="17" t="str">
-        <x:v>Four clamps in CAD; notes report mat/band electrical heaters and intended 40-in coverage</x:v>
-      </x:c>
-      <x:c r="J39" s="17" t="str">
-        <x:v>Reported</x:v>
-      </x:c>
-      <x:c r="K39" s="17" t="str">
-        <x:v>HEAT; R9</x:v>
-      </x:c>
-      <x:c r="L39" s="17" t="str">
-        <x:v>HEAT lines 16-23; R9 sheet 4</x:v>
+      <x:c r="I39" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Electrical heater footprint remains unverified. GEO-008 assumes full projected H-A span 0-1346.496215 mm for modeling only; mechanical clamps do not establish active heating.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J39" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K39" s="17" t="inlineStr">
+        <x:is>
+          <x:t>HEAT; VSEL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L39" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 lower-leg assumption; original Active heater baseline remains null</x:t>
+        </x:is>
       </x:c>
       <x:c r="M39" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -4136,17 +4671,25 @@
       <x:c r="H54" s="17" t="str">
         <x:v>Sheet 8 qualifications; model stages</x:v>
       </x:c>
-      <x:c r="I54" s="17" t="str">
-        <x:v>Heater overlap/offset and G-H path require an explicit interpretation</x:v>
-      </x:c>
-      <x:c r="J54" s="17" t="str">
-        <x:v>CAD-derived</x:v>
-      </x:c>
-      <x:c r="K54" s="17" t="str">
-        <x:v>R9</x:v>
-      </x:c>
-      <x:c r="L54" s="17" t="str">
-        <x:v>Sheets 2, 8</x:v>
+      <x:c r="I54" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Rev9 selected as provisional working geometry; main nominal ID 26.64 mm is separate from CAD null. H-A projected union is not an exact connected centerline; G-H reconstructed spline remains qualified.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J54" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K54" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VSEL; SEG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L54" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 Why H-A has a qualification; Geometry notes; CAD dimensions tab</x:t>
+        </x:is>
       </x:c>
       <x:c r="M54" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -4376,20 +4919,30 @@
       <x:c r="H59" s="17" t="str">
         <x:v>Duty definitions; VCU electrical adaptation</x:v>
       </x:c>
-      <x:c r="I59" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="J59" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="K59" s="17" t="str">
-        <x:v>None supplied</x:v>
-      </x:c>
-      <x:c r="L59" s="17" t="str">
-        <x:v>Not available</x:v>
-      </x:c>
-      <x:c r="M59" s="17" t="str">
-        <x:v>Needs information</x:v>
+      <x:c r="I59" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 assumes uniform extent over H-A projected span 1346.496215 mm. Real electrical power, spatial distribution, efficiency and heater/structure storage remain unresolved.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J59" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K59" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VSEL; HEAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L59" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-008 lower-leg modeling assumption; Thermal spans keeps installed footprint unknown</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M59" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N59" s="17" t="str">
         <x:v>Specify spatial source, meter boundary, external losses and storage without double counting.</x:v>
@@ -4568,17 +5121,23 @@
       <x:c r="H63" s="17" t="str">
         <x:v>Definitions: fixed property reference</x:v>
       </x:c>
-      <x:c r="I63" s="17" t="str">
-        <x:v>Reported 316L and insulation products; exact fluid formulation unresolved</x:v>
+      <x:c r="I63" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported 316L pipe, fiberglass candidate and calcium-aluminum-silicate strip; VMAT explicitly marks all three calibration-ineligible and unverified against installed products. Fluid formulation remains unresolved.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J63" s="17" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K63" s="17" t="str">
-        <x:v>MAT</x:v>
-      </x:c>
-      <x:c r="L63" s="17" t="str">
-        <x:v>VCU section lines 17-44</x:v>
+      <x:c r="K63" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; MAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L63" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT materials.*.provenance and calibration_eligible; Materials tab</x:t>
+        </x:is>
       </x:c>
       <x:c r="M63" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -4616,17 +5175,23 @@
       <x:c r="H64" s="17" t="str">
         <x:v>Definitions and Conventions</x:v>
       </x:c>
-      <x:c r="I64" s="17" t="str">
-        <x:v>Insulation k(T) candidate exists in notes; no correlation approved</x:v>
+      <x:c r="I64" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Nine explicit solid rho/cp/k functions transcribed from VMAT v3. Original derivations and installed-product source data remain unverified. No fluid functions imported.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J64" s="17" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K64" s="17" t="str">
-        <x:v>MAT; STEEL; PG</x:v>
-      </x:c>
-      <x:c r="L64" s="17" t="str">
-        <x:v>MAT lines 35-40; STEEL Suggested you use; PG notes</x:v>
+      <x:c r="K64" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L64" s="17" t="inlineStr">
+        <x:is>
+          <x:t>vcu_candidate_materials_v3.yaml materials.*.properties; Materials equations</x:t>
+        </x:is>
       </x:c>
       <x:c r="M64" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -4664,20 +5229,30 @@
       <x:c r="H65" s="17" t="str">
         <x:v>Definitions: property reference</x:v>
       </x:c>
-      <x:c r="I65" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="J65" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="K65" s="17" t="str">
-        <x:v>None supplied</x:v>
-      </x:c>
-      <x:c r="L65" s="17" t="str">
-        <x:v>Not available</x:v>
-      </x:c>
-      <x:c r="M65" s="17" t="str">
-        <x:v>Needs information</x:v>
+      <x:c r="I65" s="17" t="inlineStr">
+        <x:is>
+          <x:t>All imported solid functions take T in K; rho kg/m^3, cp J/(kg*K), k W/(m*K). Prop-30 mass fraction 0.30 is reported; formulation verification pending.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J65" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K65" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; PG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L65" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT properties units/coefficient_order; Fluids tab</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M65" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N65" s="17" t="str">
         <x:v>Record K versus deg C, pressure units, mass/volume fraction and output units for each function.</x:v>
@@ -4712,17 +5287,25 @@
       <x:c r="H66" s="17" t="str">
         <x:v>Property reference; temperature/condensation applicability</x:v>
       </x:c>
-      <x:c r="I66" s="17" t="str">
-        <x:v>Insulation fit is reported valid 297-533 K; not an experiment operating range</x:v>
-      </x:c>
-      <x:c r="J66" s="17" t="str">
-        <x:v>Reported</x:v>
-      </x:c>
-      <x:c r="K66" s="17" t="str">
-        <x:v>MAT</x:v>
-      </x:c>
-      <x:c r="L66" s="17" t="str">
-        <x:v>Lines 38-40</x:v>
+      <x:c r="I66" s="17" t="inlineStr">
+        <x:is>
+          <x:t>User-authorized working intervals: pipe 278.15-813 K; fiberglass 278.15-533 K; heater strip 278.15-1089 K. ADR-0033 extends all nine functions to 5 C; extrapolation is not product validation or an operating limit.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J66" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K66" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L66" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT valid_temperature_K; ADR-0033 Decision and authority</x:t>
+        </x:is>
       </x:c>
       <x:c r="M66" s="17" t="str">
         <x:v>Needs review</x:v>
@@ -4760,20 +5343,30 @@
       <x:c r="H67" s="17" t="str">
         <x:v>Proposed implementation control</x:v>
       </x:c>
-      <x:c r="I67" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="J67" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="K67" s="17" t="str">
-        <x:v>None supplied</x:v>
-      </x:c>
-      <x:c r="L67" s="17" t="str">
-        <x:v>Not available</x:v>
-      </x:c>
-      <x:c r="M67" s="17" t="str">
-        <x:v>Needs information</x:v>
+      <x:c r="I67" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT polynomial functions use ascending powers of T in K; density/cp constants as specified; all nine functions specify out_of_range: error. No fluid interpolation policy supplied.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J67" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K67" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L67" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT materials.*.properties model/coefficient_order/out_of_range</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M67" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N67" s="17" t="str">
         <x:v>Specify interpolation; reject/flag extrapolation explicitly rather than silently clipping.</x:v>
@@ -4856,20 +5449,30 @@
       <x:c r="H69" s="17" t="str">
         <x:v>Requested material-property justification</x:v>
       </x:c>
-      <x:c r="I69" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="J69" s="17" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="K69" s="17" t="str">
-        <x:v>None supplied</x:v>
-      </x:c>
-      <x:c r="L69" s="17" t="str">
-        <x:v>Not available</x:v>
-      </x:c>
-      <x:c r="M69" s="17" t="str">
-        <x:v>Needs information</x:v>
+      <x:c r="I69" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Candidate working functions supplied by user; ADR-0033 authorizes low-temperature extrapolation. Reported independent pipe comparison has no retained comparison table; package transfer does not establish independent validation.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J69" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K69" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L69" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT provenance; ADR-0033 Evidence and limits</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M69" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N69" s="17" t="str">
         <x:v>Compare candidate sources and explain selection or any deliberate mixed-source set.</x:v>
@@ -5559,7 +6162,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe3645e732ce4448"/>
+    <x:tablePart r:id="Rfe3645e732ce4448"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6508,7 +7111,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
@@ -6856,10 +7459,118 @@
         <x:v>Assistant-proposed documentation field/convention, not an approved physical fact.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VMAT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="17" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-07 v3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="17" t="inlineStr">
+        <x:is>
+          <x:t>materials.*.properties; provenance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Nine user-supplied solid-property candidates; not product verified; calibration-ineligible. Coverage wording in older provenance is superseded by VSEL.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="17" t="inlineStr">
+        <x:is>
+          <x:t>V5C</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/ADR-0033-vcu-solid-properties-5c.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="17" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-07 accepted working-range decision</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Decision and authority; Evidence and limits</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="17" t="inlineStr">
+        <x:is>
+          <x:t>User authorizes working extrapolation to 5 C, not source/product validation or an operating limit.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VSEL</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="17" t="inlineStr">
+        <x:is>
+          <x:t>2026-10-14 provisional working selection</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="17" t="inlineStr">
+        <x:is>
+          <x:t>User direction and interpretation; Why H-A has a qualification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Dated working geometry/installation choices; historical run dates, tips and electrical footprint unresolved.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VINS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="17" t="inlineStr">
+        <x:is>
+          <x:t>v5 2026-10-07, amended by VSEL for Rev9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="17" t="inlineStr">
+        <x:is>
+          <x:t>coverage; contact; regions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Regional thickness estimates/contact assumption; exact transitions and installed construction unverified. VSEL is later controlling top-leg evidence.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd789b6a13c34804"/>
+    <x:tablePart r:id="Rbd789b6a13c34804"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7042,8 +7753,16 @@
       <x:c r="G6" s="33" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="H6" s="33"/>
-      <x:c r="I6" s="33"/>
+      <x:c r="H6" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / non_heater_main_pipe</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported approximate 50.8 mm fiberglass candidate; exact transitions/gaps and bare STC contacts unresolved. Whole-region coverage remains Unknown.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
       <x:c r="A7" s="32" t="str">
@@ -7076,16 +7795,28 @@
       <x:c r="C8" s="32" t="str">
         <x:v>Segment start to Complete jacket start</x:v>
       </x:c>
-      <x:c r="D8" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D8" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Bare</x:t>
+        </x:is>
       </x:c>
       <x:c r="E8" s="33"/>
       <x:c r="F8" s="34"/>
-      <x:c r="G8" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H8" s="33"/>
-      <x:c r="I8" s="33"/>
+      <x:c r="G8" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="33" t="inlineStr">
+        <x:is>
+          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="32" t="str">
@@ -7097,17 +7828,27 @@
       <x:c r="C9" s="32" t="str">
         <x:v>Complete jacket start to Complete jacket end</x:v>
       </x:c>
-      <x:c r="D9" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D9" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Bare</x:t>
+        </x:is>
       </x:c>
       <x:c r="E9" s="33"/>
       <x:c r="F9" s="34"/>
-      <x:c r="G9" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H9" s="33"/>
-      <x:c r="I9" s="33" t="str">
-        <x:v>Identify the insulated surface, especially jacket exterior versus pipe.</x:v>
+      <x:c r="G9" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" s="33" t="inlineStr">
+        <x:is>
+          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -7120,16 +7861,28 @@
       <x:c r="C10" s="32" t="str">
         <x:v>Complete jacket end to segment end</x:v>
       </x:c>
-      <x:c r="D10" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D10" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Bare</x:t>
+        </x:is>
       </x:c>
       <x:c r="E10" s="33"/>
       <x:c r="F10" s="34"/>
-      <x:c r="G10" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H10" s="33"/>
-      <x:c r="I10" s="33"/>
+      <x:c r="G10" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" s="33" t="inlineStr">
+        <x:is>
+          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="32" t="str">
@@ -7170,8 +7923,16 @@
       <x:c r="G12" s="33" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="H12" s="33"/>
-      <x:c r="I12" s="33"/>
+      <x:c r="H12" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / non_heater_main_pipe</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported approximate 50.8 mm fiberglass candidate; exact transitions/gaps and bare STC contacts unresolved. Whole-region coverage remains Unknown.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
       <x:c r="A13" s="32" t="str">
@@ -7212,8 +7973,16 @@
       <x:c r="G14" s="33" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="H14" s="33"/>
-      <x:c r="I14" s="33"/>
+      <x:c r="H14" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / heater_leg</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported approximate 6.35 mm calcium-aluminum-silicate strip only; exact coverage and installed stack unverified. Whole-region coverage remains Unknown.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
       <x:c r="A15" s="32" t="str">
@@ -7422,8 +8191,10 @@
       <x:c r="M6" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N6" s="8" t="str">
-        <x:v>Continuous straight axis</x:v>
+      <x:c r="N6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Continuous straight axis; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
@@ -7458,8 +8229,10 @@
       <x:c r="M7" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N7" s="8" t="str">
-        <x:v>Exact analytical torus centerline arc</x:v>
+      <x:c r="N7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Exact analytical torus centerline arc; CAD torus radius 57.150000 mm, angle 100.800000 deg, arc 100.543531 mm. Diagram connector remains schematic.; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
@@ -7494,8 +8267,10 @@
       <x:c r="M8" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N8" s="8" t="str">
-        <x:v>Continuous straight axis</x:v>
+      <x:c r="N8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Continuous straight axis; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
@@ -7530,8 +8305,10 @@
       <x:c r="M9" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N9" s="8" t="str">
-        <x:v>Exact analytical torus centerline arc</x:v>
+      <x:c r="N9" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Exact analytical torus centerline arc; CAD torus radius 57.150000 mm, angle 79.200000 deg, arc 78.998489 mm. Diagram connector remains schematic.; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10" ht="26" customHeight="1">
@@ -7566,8 +8343,10 @@
       <x:c r="M10" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N10" s="8" t="str">
-        <x:v>Continuous straight axis</x:v>
+      <x:c r="N10" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Continuous straight axis; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
@@ -7602,8 +8381,10 @@
       <x:c r="M11" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N11" s="8" t="str">
-        <x:v>Endpoint chord exact; recovered spline spine qualified by endpoint residuals</x:v>
+      <x:c r="N11" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Endpoint chord exact; recovered spline spine qualified by endpoint residuals; recovered spine 98.265651493 mm is qualified; exact centerline length remains unknown.; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12" ht="26" customHeight="1">
@@ -7638,8 +8419,10 @@
       <x:c r="M12" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N12" s="8" t="str">
-        <x:v>Projected endpoint-to-endpoint axial span; overlapping offset pieces retained, no healed centerline</x:v>
+      <x:c r="N12" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Projected endpoint-to-endpoint axial span; overlapping offset pieces retained, no healed centerline; axis sum 1353.698559747 mm, projected overlap 7.202344895 mm, transverse offset 0.151551091 mm. VSEL full-span heating is a modeling assumption; installed footprint unknown.; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13" ht="26" customHeight="1">
@@ -7674,8 +8457,10 @@
       <x:c r="M13" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 1-3</x:v>
       </x:c>
-      <x:c r="N13" s="8" t="str">
-        <x:v>Exact analytical torus centerline arc</x:v>
+      <x:c r="N13" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Exact analytical torus centerline arc; CAD torus radius 57.150000 mm, angle 79.200000 deg, arc 78.998489 mm. Diagram connector remains schematic.; portable SEG CSV in support/evidence/2026-10-16_CFG-001_vcu_references/VCU_Rev9_Segments.csv.</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9484,19 +10269,39 @@
       <x:c r="C6" s="8" t="str">
         <x:v>rho, cp, k</x:v>
       </x:c>
-      <x:c r="D6" s="8"/>
-      <x:c r="E6" s="8"/>
-      <x:c r="F6" s="8"/>
-      <x:c r="G6" s="8"/>
+      <x:c r="D6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho(T) = (8066.715) + (-0.398373)*T; cp(T) = (279.256) + (0.732165)*T + (-0.000459146)*T^2; k(T) = (9.248) + (0.01571)*T</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>T in kelvin (K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho: kg/m^3; cp: J/(kg*K); k: W/(m*K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Working use only: 278.15-813 K; lower extension authorized 2026-10-07, not product validation. Pressure domain not supplied.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="H6" s="8"/>
-      <x:c r="I6" s="8" t="str">
-        <x:v>Reconcile candidate correlations and installed specification.</x:v>
+      <x:c r="I6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J6" s="8" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K6" s="8" t="str">
-        <x:v>1.2 Main Material Props.md; 1.2.2 Steel Pipe Properties.md</x:v>
+      <x:c r="K6" s="8" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_pipe_316l_user_candidate_v1.properties</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="26" customHeight="1">
@@ -9509,19 +10314,39 @@
       <x:c r="C7" s="8" t="str">
         <x:v>rho, cp, k</x:v>
       </x:c>
-      <x:c r="D7" s="8"/>
-      <x:c r="E7" s="8"/>
-      <x:c r="F7" s="8"/>
-      <x:c r="G7" s="8"/>
+      <x:c r="D7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho(T) = 72.08; cp(T) = 840.0; k(T) = (0.0678938) + (-0.000289613)*T + (5.84142e-07)*T^2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>T in kelvin (K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho: kg/m^3; cp: J/(kg*K); k: W/(m*K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Working use only: 278.15-533 K; lower extension authorized 2026-10-07, not product validation. Pressure domain not supplied.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="H7" s="8"/>
-      <x:c r="I7" s="8" t="str">
-        <x:v>Confirm installed layers and original product evidence.</x:v>
+      <x:c r="I7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 50.8 mm thickness is a provisional regional estimate, not a measurement; old library coverage wording is superseded by GEO-008.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J7" s="8" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K7" s="8" t="str">
-        <x:v>1.2 Main Material Props.md</x:v>
+      <x:c r="K7" s="8" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_main_fiberglass_user_candidate_v1.properties</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="26" customHeight="1">
@@ -9534,19 +10359,39 @@
       <x:c r="C8" s="8" t="str">
         <x:v>rho, cp, k</x:v>
       </x:c>
-      <x:c r="D8" s="8"/>
-      <x:c r="E8" s="8"/>
-      <x:c r="F8" s="8"/>
-      <x:c r="G8" s="8"/>
+      <x:c r="D8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho(T) = 560.65; cp(T) = (709.85) + (0.3075)*T; k(T) = (0.101729) + (-0.000201327)*T + (3.21455e-07)*T^2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>T in kelvin (K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>rho: kg/m^3; cp: J/(kg*K); k: W/(m*K)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Working use only: 278.15-1089 K; lower extension authorized 2026-10-07, not product validation. Pressure domain not supplied.</x:t>
+        </x:is>
+      </x:c>
       <x:c r="H8" s="8"/>
-      <x:c r="I8" s="8" t="str">
-        <x:v>Confirm installed stack and contacts.</x:v>
+      <x:c r="I8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 6.35 mm strip only on heater leg; installed layer order and contacts unverified.</x:t>
+        </x:is>
       </x:c>
       <x:c r="J8" s="8" t="str">
         <x:v>Reported</x:v>
       </x:c>
-      <x:c r="K8" s="8" t="str">
-        <x:v>1.2 Main Material Props.md</x:v>
+      <x:c r="K8" s="8" t="inlineStr">
+        <x:is>
+          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_heater_cas_strip_user_candidate_v1.properties</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9" ht="26" customHeight="1">
@@ -9860,6 +10705,90 @@
       <x:c r="G14" s="8"/>
       <x:c r="H14" s="8" t="str">
         <x:v>Unknown</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Main nominal bore</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>CAD bore absent</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Reference working nominal ID 26.64 mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Nominal ID 26.64 mm candidate; local restrictions need explicit treatment</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>VSEL; DIA. Rounded nominal selection; not a CAD bore or installed measurement. Geometry ID cells remain null.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Actual bore and local spool restrictions unresolved.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Computational + experimental review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Heater spatial extent</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Electrical footprint unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Reference assumption: H-A 0 to 1346.496215 mm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Same projected-span candidate; connected geometry and heat source require review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>VSEL. Full lower-leg heating assumption only; active baseline spans remain null.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Electrical power split, storage, losses and footprint unresolved.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Computational + experimental review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Modeling assumption</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Correct VCU upper corners and LF-01 to covered per user clarification
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -1032,7 +1032,7 @@
       </x:c>
       <x:c r="B7" s="9" t="inlineStr">
         <x:is>
-          <x:t>VCU-REV9-DRAFT-004</x:t>
+          <x:t>VCU-REV9-DRAFT-005</x:t>
         </x:is>
       </x:c>
       <x:c r="C7" s="8" t="str">
@@ -1210,7 +1210,7 @@
       </x:c>
       <x:c r="B23" s="9" t="inlineStr">
         <x:is>
-          <x:t>CFG-001: VCU Rev9 component dimensions; nine solid-property candidate functions with SI units and working domains; portable source copies; dated nominal-ID, insulation and heater assumptions in evidence records. Physical installation and approval remain open.</x:t>
+          <x:t>GEO-009: entire covered top-left C-D and top-right E-F corners Insulated; LF-01 locally covered, per Andres Fierro 2026-10-16. Model regional insulation v6 and Rev9 working selection v2 agree. Other coverage, numerical geometry and historical evidence unchanged.</x:t>
         </x:is>
       </x:c>
       <x:c r="C23" s="9" t="str">
@@ -3017,7 +3017,7 @@
       </x:c>
       <x:c r="I20" s="17" t="inlineStr">
         <x:is>
-          <x:t>GEO-008 reports whole top D-E uninsulated; all STCs contact bare pipe locally. Remaining transition endpoints unknown. Older full-loop coverage text is superseded.</x:t>
+          <x:t>User 2026-10-16: entire C-D/E-F upper corners insulated; LF-01 locally covered. Top D-E remains bare. Remaining vertical cutbacks and LF-01 coverage extent unknown.</x:t>
         </x:is>
       </x:c>
       <x:c r="J20" s="17" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </x:c>
       <x:c r="K20" s="17" t="inlineStr">
         <x:is>
-          <x:t>VSEL; VINS</x:t>
+          <x:t>VSEL; VTOP</x:t>
         </x:is>
       </x:c>
       <x:c r="L20" s="17" t="inlineStr">
         <x:is>
-          <x:t>GEO-008 User direction and interpretation; insulation.yaml coverage</x:t>
+          <x:t>VTOP direct user clarification; Insulation regions INS-02/06; Sensors LF-01; regional model v6</x:t>
         </x:is>
       </x:c>
       <x:c r="M20" s="17" t="inlineStr">
@@ -7567,6 +7567,33 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VTOP</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-009_covered_top_corners/USER_CLARIFICATION.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Direct user clarification 2026-10-16; model regional v6 / Rev9 working v2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Whole C-D / E-F corners; LF-01 local exposure</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported by user; no independent survey, optical extent, covered extent or historical run dates supplied.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
@@ -7774,16 +7801,28 @@
       <x:c r="C7" s="32" t="str">
         <x:v>Full schematic corner</x:v>
       </x:c>
-      <x:c r="D7" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D7" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
       </x:c>
       <x:c r="E7" s="33"/>
       <x:c r="F7" s="34"/>
-      <x:c r="G7" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H7" s="33"/>
-      <x:c r="I7" s="33"/>
+      <x:c r="G7" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-009_covered_top_corners/USER_CLARIFICATION.md / entire covered top-left C-D and top-right E-F corners</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Entire corner insulated per corrected Andres Fierro statement 2026-10-16. Installed product and thickness unmeasured; model fiberglass estimate remains provisional.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="32" t="str">
@@ -7894,16 +7933,28 @@
       <x:c r="C11" s="32" t="str">
         <x:v>Full schematic corner</x:v>
       </x:c>
-      <x:c r="D11" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D11" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
       </x:c>
       <x:c r="E11" s="33"/>
       <x:c r="F11" s="34"/>
-      <x:c r="G11" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H11" s="33"/>
-      <x:c r="I11" s="33"/>
+      <x:c r="G11" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-009_covered_top_corners/USER_CLARIFICATION.md / entire covered top-left C-D and top-right E-F corners</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Entire corner insulated per corrected Andres Fierro statement 2026-10-16. Installed product and thickness unmeasured; model fiberglass estimate remains provisional.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
       <x:c r="A12" s="32" t="str">
@@ -8748,8 +8799,10 @@
       <x:c r="K10" s="8" t="str">
         <x:v>VCU-R9-E01 (2026-10-08) sheets 5-7</x:v>
       </x:c>
-      <x:c r="L10" s="8" t="str">
-        <x:v>Actual sensing location and channel mapping unverified.</x:v>
+      <x:c r="L10" s="8" t="inlineStr">
+        <x:is>
+          <x:t>Actual sensing location and channel mapping unverified. User report 2026-10-16 (VTOP): LF-01 is covered locally. CAD mount reference lies on upcomer 61.113919 mm below C; covered extent, optical extent and DAQ mapping remain unknown.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">

</xml_diff>

<commit_message>
Synchronize all VCU insulation regions and reported thicknesses
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -1032,7 +1032,7 @@
       </x:c>
       <x:c r="B7" s="9" t="inlineStr">
         <x:is>
-          <x:t>VCU-REV9-DRAFT-005</x:t>
+          <x:t>VCU-REV9-DRAFT-006</x:t>
         </x:is>
       </x:c>
       <x:c r="C7" s="8" t="str">
@@ -1210,7 +1210,7 @@
       </x:c>
       <x:c r="B23" s="9" t="inlineStr">
         <x:is>
-          <x:t>GEO-009: entire covered top-left C-D and top-right E-F corners Insulated; LF-01 locally covered, per Andres Fierro 2026-10-16. Model regional insulation v6 and Rev9 working selection v2 agree. Other coverage, numerical geometry and historical evidence unchanged.</x:t>
+          <x:t>GEO-010: all ten insulation regions synchronized: six ordinary-pipe fiberglass regions about 50.8 mm; heater ceramic strip only about 6.35 mm; three top D-E partitions Bare. Coverage Reported; thicknesses approximate estimates. LF-01 remains covered.</x:t>
         </x:is>
       </x:c>
       <x:c r="C23" s="9" t="str">
@@ -2909,24 +2909,28 @@
       </x:c>
       <x:c r="I18" s="17" t="inlineStr">
         <x:is>
-          <x:t>Reported fiberglass main insulation and calcium-aluminum-silicate heater strip. VINS v5 specifies regional candidates; product/installation evidence unresolved.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J18" s="17" t="str">
-        <x:v>Reported</x:v>
+          <x:t>Ordinary main piping (upcomer/downcomer and four corners): fiberglass MAIN-INS; heater: calcium-aluminum-silicate HEATER-INS strip only, no additional fiberglass.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
       </x:c>
       <x:c r="K18" s="17" t="inlineStr">
         <x:is>
-          <x:t>MAT; VINS</x:t>
+          <x:t>VREG; VTOP</x:t>
         </x:is>
       </x:c>
       <x:c r="L18" s="17" t="inlineStr">
         <x:is>
-          <x:t>Materials; insulation.yaml regions; source copies in support/evidence/2026-10-16_CFG-001_vcu_references</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M18" s="17" t="str">
-        <x:v>Needs review</x:v>
+          <x:t>VREG regional YAML and ADR-0025/0026; VTOP corner/LF-01 correction; user reaffirmation 2026-10-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M18" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N18" s="17" t="str">
         <x:v>Which product and layers are installed on this exact segment?</x:v>
@@ -2963,24 +2967,28 @@
       </x:c>
       <x:c r="I19" s="17" t="inlineStr">
         <x:is>
-          <x:t>Approximate regional estimates: ordinary insulated pipe 50.8 mm fiberglass; heater 6.35 mm strip only. Top D-E is bare per GEO-008. Not measured thicknesses.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J19" s="17" t="str">
-        <x:v>Reported</x:v>
+          <x:t>Reported estimates: ordinary insulated regions 50.8 mm (2 in); heater strip 6.35 mm (1/4 in). Not installed thickness measurements.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
       </x:c>
       <x:c r="K19" s="17" t="inlineStr">
         <x:is>
-          <x:t>VINS; VSEL</x:t>
+          <x:t>VREG; VTOP</x:t>
         </x:is>
       </x:c>
       <x:c r="L19" s="17" t="inlineStr">
         <x:is>
-          <x:t>insulation.yaml regions.non_heater_main_pipe and heater_leg; GEO-008 top-leg qualification</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M19" s="17" t="str">
-        <x:v>Needs review</x:v>
+          <x:t>VREG regional YAML and ADR-0025/0026; VTOP corner/LF-01 correction; user reaffirmation 2026-10-16</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="M19" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Needs review</x:t>
+        </x:is>
       </x:c>
       <x:c r="N19" s="17" t="str">
         <x:v>Measure each layer; do not apply either value everywhere.</x:v>
@@ -3017,7 +3025,7 @@
       </x:c>
       <x:c r="I20" s="17" t="inlineStr">
         <x:is>
-          <x:t>User 2026-10-16: entire C-D/E-F upper corners insulated; LF-01 locally covered. Top D-E remains bare. Remaining vertical cutbacks and LF-01 coverage extent unknown.</x:t>
+          <x:t>Reported coverage known for all ten regions: upcomer/downcomer, four corners and heater insulated; pre-cooler/jacket/post-cooler D-E bare. LF-01 covered. Exact local contacts and transitions remain open.</x:t>
         </x:is>
       </x:c>
       <x:c r="J20" s="17" t="inlineStr">
@@ -3027,12 +3035,12 @@
       </x:c>
       <x:c r="K20" s="17" t="inlineStr">
         <x:is>
-          <x:t>VSEL; VTOP</x:t>
+          <x:t>VREG; VTOP</x:t>
         </x:is>
       </x:c>
       <x:c r="L20" s="17" t="inlineStr">
         <x:is>
-          <x:t>VTOP direct user clarification; Insulation regions INS-02/06; Sensors LF-01; regional model v6</x:t>
+          <x:t>VREG regional YAML and ADR-0025/0026; VTOP corner/LF-01 correction; user reaffirmation 2026-10-16</x:t>
         </x:is>
       </x:c>
       <x:c r="M20" s="17" t="inlineStr">
@@ -7594,6 +7602,33 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="17" t="inlineStr">
+        <x:is>
+          <x:t>VREG</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="17" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/README.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="17" t="inlineStr">
+        <x:is>
+          <x:t>GEO-010 2026-10-16; regional v7 / working v3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="17" t="inlineStr">
+        <x:is>
+          <x:t>region_assignments.json; insulation.yaml; ADR-0025/0026; USER_CONFIRMATION.md</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="17" t="inlineStr">
+        <x:is>
+          <x:t>Reported coverage and approximate thickness estimates; product/fit validation, installed surveys and historical applicability remain separate.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
@@ -7772,22 +7807,32 @@
       <x:c r="C6" s="32" t="str">
         <x:v>Full segment</x:v>
       </x:c>
-      <x:c r="D6" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E6" s="33"/>
-      <x:c r="F6" s="34"/>
-      <x:c r="G6" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D6" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="G6" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
       </x:c>
       <x:c r="H6" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / non_heater_main_pipe</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I6" s="33" t="inlineStr">
         <x:is>
-          <x:t>Reported approximate 50.8 mm fiberglass candidate; exact transitions/gaps and bare STC contacts unresolved. Whole-region coverage remains Unknown.</x:t>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7806,8 +7851,14 @@
           <x:t>Insulated</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" s="33"/>
-      <x:c r="F7" s="34"/>
+      <x:c r="E7" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
       <x:c r="G7" s="33" t="inlineStr">
         <x:is>
           <x:t>Reported</x:t>
@@ -7815,12 +7866,12 @@
       </x:c>
       <x:c r="H7" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_GEO-009_covered_top_corners/USER_CLARIFICATION.md / entire covered top-left C-D and top-right E-F corners</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I7" s="33" t="inlineStr">
         <x:is>
-          <x:t>Entire corner insulated per corrected Andres Fierro statement 2026-10-16. Installed product and thickness unmeasured; model fiberglass estimate remains provisional.</x:t>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7848,12 +7899,12 @@
       </x:c>
       <x:c r="H8" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I8" s="33" t="inlineStr">
         <x:is>
-          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+          <x:t>Reported straight top D-E bare, GEO-008 retained; water jacket remains present.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7881,12 +7932,12 @@
       </x:c>
       <x:c r="H9" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I9" s="33" t="inlineStr">
         <x:is>
-          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+          <x:t>Reported straight top D-E bare, GEO-008 retained; water jacket remains present.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7914,12 +7965,12 @@
       </x:c>
       <x:c r="H10" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/2026-10-14_GEO-008_rev9_working_selection.md / whole top D-E leg</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I10" s="33" t="inlineStr">
         <x:is>
-          <x:t>October 14 user-reported working installation; not independently surveyed. Water jacket remains present; Bare does not imply room-air exposure beneath jacket.</x:t>
+          <x:t>Reported straight top D-E bare, GEO-008 retained; water jacket remains present.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7938,8 +7989,14 @@
           <x:t>Insulated</x:t>
         </x:is>
       </x:c>
-      <x:c r="E11" s="33"/>
-      <x:c r="F11" s="34"/>
+      <x:c r="E11" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
       <x:c r="G11" s="33" t="inlineStr">
         <x:is>
           <x:t>Reported</x:t>
@@ -7947,12 +8004,12 @@
       </x:c>
       <x:c r="H11" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_GEO-009_covered_top_corners/USER_CLARIFICATION.md / entire covered top-left C-D and top-right E-F corners</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I11" s="33" t="inlineStr">
         <x:is>
-          <x:t>Entire corner insulated per corrected Andres Fierro statement 2026-10-16. Installed product and thickness unmeasured; model fiberglass estimate remains provisional.</x:t>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7966,22 +8023,32 @@
       <x:c r="C12" s="32" t="str">
         <x:v>Full segment</x:v>
       </x:c>
-      <x:c r="D12" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E12" s="33"/>
-      <x:c r="F12" s="34"/>
-      <x:c r="G12" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D12" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="G12" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
       </x:c>
       <x:c r="H12" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / non_heater_main_pipe</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I12" s="33" t="inlineStr">
         <x:is>
-          <x:t>Reported approximate 50.8 mm fiberglass candidate; exact transitions/gaps and bare STC contacts unresolved. Whole-region coverage remains Unknown.</x:t>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7995,16 +8062,34 @@
       <x:c r="C13" s="32" t="str">
         <x:v>Full schematic corner</x:v>
       </x:c>
-      <x:c r="D13" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E13" s="33"/>
-      <x:c r="F13" s="34"/>
-      <x:c r="G13" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H13" s="33"/>
-      <x:c r="I13" s="33"/>
+      <x:c r="D13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="G13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
       <x:c r="A14" s="32" t="str">
@@ -8016,22 +8101,32 @@
       <x:c r="C14" s="32" t="str">
         <x:v>Full segment</x:v>
       </x:c>
-      <x:c r="D14" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E14" s="33"/>
-      <x:c r="F14" s="34"/>
-      <x:c r="G14" s="33" t="str">
-        <x:v>Unknown</x:v>
+      <x:c r="D14" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="33" t="inlineStr">
+        <x:is>
+          <x:t>HEATER-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="34">
+        <x:v>6.35</x:v>
+      </x:c>
+      <x:c r="G14" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
       </x:c>
       <x:c r="H14" s="33" t="inlineStr">
         <x:is>
-          <x:t>support/evidence/2026-10-16_CFG-001_vcu_references/insulation.yaml / heater_leg</x:t>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
         </x:is>
       </x:c>
       <x:c r="I14" s="33" t="inlineStr">
         <x:is>
-          <x:t>Reported approximate 6.35 mm calcium-aluminum-silicate strip only; exact coverage and installed stack unverified. Whole-region coverage remains Unknown.</x:t>
+          <x:t>Reported heater insulation: approximately 1/4 in calcium-aluminum-silicate ceramic-fiber strip only; no extra fiberglass. Thickness is an estimate, not measured.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -8045,16 +8140,34 @@
       <x:c r="C15" s="32" t="str">
         <x:v>Full schematic corner</x:v>
       </x:c>
-      <x:c r="D15" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E15" s="33"/>
-      <x:c r="F15" s="34"/>
-      <x:c r="G15" s="33" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="H15" s="33"/>
-      <x:c r="I15" s="33"/>
+      <x:c r="D15" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Insulated</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="33" t="inlineStr">
+        <x:is>
+          <x:t>MAIN-INS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="34">
+        <x:v>50.8</x:v>
+      </x:c>
+      <x:c r="G15" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" s="33" t="inlineStr">
+        <x:is>
+          <x:t>support/evidence/2026-10-16_GEO-010_regional_insulation_sync/insulation.yaml / regions; VREG; VCU-007/008 and GEO-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I15" s="33" t="inlineStr">
+        <x:is>
+          <x:t>Reported ordinary main-pipe fiberglass assignment, approximately 2 in; regional model candidate, not installed product/thickness validation. Local STC contacts/transition details remain separate.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -10390,7 +10503,7 @@
       <x:c r="H7" s="8"/>
       <x:c r="I7" s="8" t="inlineStr">
         <x:is>
-          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 50.8 mm thickness is a provisional regional estimate, not a measurement; old library coverage wording is superseded by GEO-008.</x:t>
+          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 50.8 mm thickness is a provisional regional estimate, not a measurement; old library coverage wording is superseded by GEO-008. Assigned to upcomer, downcomer and all four corners; approximately 50.8 mm fiberglass. Reported assignment; exact product and thickness remain unverified.</x:t>
         </x:is>
       </x:c>
       <x:c r="J7" s="8" t="str">
@@ -10398,7 +10511,7 @@
       </x:c>
       <x:c r="K7" s="8" t="inlineStr">
         <x:is>
-          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_main_fiberglass_user_candidate_v1.properties</x:t>
+          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_main_fiberglass_user_candidate_v1.properties; VREG</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -10435,7 +10548,7 @@
       <x:c r="H8" s="8"/>
       <x:c r="I8" s="8" t="inlineStr">
         <x:is>
-          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 6.35 mm strip only on heater leg; installed layer order and contacts unverified.</x:t>
+          <x:t>Reported user-supplied candidate; calibration_eligible=false. No original fit derivation, installed-product verification or uncertainty supplied. Below original lower bounds (pipe/strip 293 K, fiberglass k 297 K) is user-authorized extrapolation per ADR-0033; not a source-validated range. Outside working range: error. Approximate 6.35 mm strip only on heater leg; installed layer order and contacts unverified. Assigned to straight heater only; approximately 6.35 mm ceramic strip; no extra fiberglass. Reported assignment; exact product and thickness remain unverified.</x:t>
         </x:is>
       </x:c>
       <x:c r="J8" s="8" t="str">
@@ -10443,7 +10556,7 @@
       </x:c>
       <x:c r="K8" s="8" t="inlineStr">
         <x:is>
-          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_heater_cas_strip_user_candidate_v1.properties</x:t>
+          <x:t>VMAT; V5C; support/evidence/2026-10-16_CFG-001_vcu_references/vcu_candidate_materials_v3.yaml / materials.vcu_heater_cas_strip_user_candidate_v1.properties; VREG</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -11114,14 +11227,20 @@
       <x:c r="B13" s="17" t="str">
         <x:v>Insulation product and layer order</x:v>
       </x:c>
-      <x:c r="C13" s="18" t="str">
-        <x:v>Most piping: fiberglass, reported 5556K73</x:v>
-      </x:c>
-      <x:c r="D13" s="18" t="str">
-        <x:v>Reported</x:v>
-      </x:c>
-      <x:c r="E13" s="18" t="str">
-        <x:v>MAT lines 29-35</x:v>
+      <x:c r="C13" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported fiberglass MAIN-INS on upcomer; heater uses distinct ceramic strip only.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VREG; user reaffirmation 2026-10-16</x:t>
+        </x:is>
       </x:c>
       <x:c r="F13" s="19"/>
       <x:c r="G13" s="19"/>
@@ -11137,14 +11256,20 @@
       <x:c r="B14" s="17" t="str">
         <x:v>Thickness of each layer (mm)</x:v>
       </x:c>
-      <x:c r="C14" s="18" t="str">
-        <x:v>About 2 in for most main piping; this segment unverified</x:v>
-      </x:c>
-      <x:c r="D14" s="18" t="str">
-        <x:v>Reported</x:v>
-      </x:c>
-      <x:c r="E14" s="18" t="str">
-        <x:v>MAT lines 29-35</x:v>
+      <x:c r="C14" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Upcomer: reported approximate 50.8 mm fiberglass; estimate, not measurement.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VREG; user reaffirmation 2026-10-16</x:t>
+        </x:is>
       </x:c>
       <x:c r="F14" s="19"/>
       <x:c r="G14" s="19"/>
@@ -11160,14 +11285,20 @@
       <x:c r="B15" s="17" t="str">
         <x:v>Coverage, gaps and condition</x:v>
       </x:c>
-      <x:c r="C15" s="18" t="str">
-        <x:v>Unknown for this exact segment</x:v>
-      </x:c>
-      <x:c r="D15" s="18" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="E15" s="18" t="str">
-        <x:v>P0 geometry/configuration request</x:v>
+      <x:c r="C15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Upcomer insulated per documented assignment and user reaffirmation; exact gaps/condition unmeasured.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>Reported</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="18" t="inlineStr">
+        <x:is>
+          <x:t>VREG; user reaffirmation 2026-10-16</x:t>
+        </x:is>
       </x:c>
       <x:c r="F15" s="19"/>
       <x:c r="G15" s="19"/>

</xml_diff>

<commit_message>
Leave workbook preparer fields blank
</commit_message>
<xml_diff>
--- a/VCU_inputs.xlsx
+++ b/VCU_inputs.xlsx
@@ -2549,11 +2549,7 @@
       <x:c r="A16" s="8" t="str">
         <x:v>Prepared by</x:v>
       </x:c>
-      <x:c r="B16" s="9" t="inlineStr">
-        <x:is>
-          <x:t>Codex / agent-root-cfg002; requested by Andres Fierro</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="B16" s="9"/>
       <x:c r="C16" s="8" t="str">
         <x:v>Enter name.</x:v>
       </x:c>

</xml_diff>